<commit_message>
Sync planning SharePoint : S20
</commit_message>
<xml_diff>
--- a/Plannings 2026 S20.xlsx
+++ b/Plannings 2026 S20.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D76AC588-95F3-4345-92E4-96684B0CB1EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{D76AC588-95F3-4345-92E4-96684B0CB1EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2A9CE38-A8D2-4D4D-8634-2C2CEF98AAD1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="106">
   <si>
     <t>Planning des salariés du 11/05/2026 au 17/05/2026</t>
   </si>
@@ -349,7 +349,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[h]:mm"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -438,6 +438,12 @@
     <font>
       <sz val="8"/>
       <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color indexed="8"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -772,7 +778,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -953,6 +959,9 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4622,6 +4631,50 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2342029" y="5636559"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="91" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F0A3FFB-1423-45E2-B0B1-8A80A2C86894}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7026088" y="3316941"/>
           <a:ext cx="123825" cy="123825"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5282,7 +5335,9 @@
       <c r="A18" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="21"/>
+      <c r="B18" s="21" t="s">
+        <v>13</v>
+      </c>
       <c r="C18" s="21"/>
       <c r="D18" s="21" t="s">
         <v>13</v>
@@ -5296,7 +5351,9 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="27"/>
-      <c r="B19" s="1"/>
+      <c r="B19" s="62" t="s">
+        <v>68</v>
+      </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1" t="s">
         <v>35</v>
@@ -6786,13 +6843,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5E0D53BC-C34C-4902-9CAE-E951C8911F64}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3B0DD343-E130-45B5-84B4-EBCC15E4C2EF}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FA22322-5C77-4CB0-93E0-631958536DF1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BE0FF401-2928-43D9-8A98-35A81B038ECB}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5ED5375D-3A3C-4A2A-96C0-A18320FFF873}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6003F7E4-418D-4F95-AF6D-767ABA8B20CF}"/>
 </file>
</xml_diff>